<commit_message>
simulations page ready for review
</commit_message>
<xml_diff>
--- a/CasesAFR/Material_Streams_1.1.xlsx
+++ b/CasesAFR/Material_Streams_1.1.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afsalem\Documents\GitHub\Senior_Project_Dashboard\CasesAFR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B6EF7C-9CEA-4CF6-8FA1-0868D4C92FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A39663-ED77-43DC-B88E-99DBB026E358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2920" yWindow="2920" windowWidth="14400" windowHeight="8260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Compositions" sheetId="2" r:id="rId1"/>
-    <sheet name="Material Streams" sheetId="3" r:id="rId2"/>
+    <sheet name="Material Streams" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Unit</t>
   </si>
@@ -64,46 +63,7 @@
     <t>Final Product</t>
   </si>
   <si>
-    <t>Comp Mole Frac (Methane)</t>
-  </si>
-  <si>
     <t/>
-  </si>
-  <si>
-    <t>Comp Mole Frac (Propane)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (i-Pentane)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (i-Butane)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (Ethane)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (CO)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (CO2)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (H2O)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (Hydrogen)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (NO2)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (NO)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (Oxygen)</t>
-  </si>
-  <si>
-    <t>Comp Mole Frac (Nitrogen)</t>
   </si>
   <si>
     <t>Vapour Fraction</t>
@@ -1010,473 +970,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.1796875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1">
-        <v>9.5072096913784685E-19</v>
-      </c>
-      <c r="D2" s="1">
-        <v>9.5072096913784685E-19</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <v>9.5072096913784685E-19</v>
-      </c>
-      <c r="G2" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="H2" s="1">
-        <v>9.5072096913784685E-19</v>
-      </c>
-      <c r="I2" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="J2" s="1">
-        <v>9.5072096913784685E-19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="1">
-        <v>8.7366849838987302E-39</v>
-      </c>
-      <c r="D3" s="1">
-        <v>8.7366849838987302E-39</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
-        <v>8.7366849838987302E-39</v>
-      </c>
-      <c r="G3" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>8.7366849838987302E-39</v>
-      </c>
-      <c r="I3" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="J3" s="1">
-        <v>8.7366849838987302E-39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="4">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1.4449312193921702E-39</v>
-      </c>
-      <c r="D4" s="1">
-        <v>1.4449312193921702E-39</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1.4449312193921702E-39</v>
-      </c>
-      <c r="G4" s="4">
-        <v>0.02</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1.4449312193921702E-39</v>
-      </c>
-      <c r="I4" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="J4" s="1">
-        <v>1.4449312193921702E-39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="4">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1.5379042423001772E-39</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1.5379042423001772E-39</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1">
-        <v>1.5379042423001772E-39</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0.01</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1.5379042423001772E-39</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="J5" s="1">
-        <v>1.5379042423001772E-39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="4">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1">
-        <v>7.5288132071059452E-36</v>
-      </c>
-      <c r="D6" s="1">
-        <v>7.5288132071059466E-36</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1">
-        <v>7.5288132071059452E-36</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="H6" s="1">
-        <v>7.5288132071059452E-36</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="J6" s="1">
-        <v>7.5288132071059466E-36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="4">
-        <v>0</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1.3946280165394675E-3</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1.3946280165394675E-3</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1">
-        <v>1.3946280165394675E-3</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
-        <v>1.3946280165394675E-3</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0</v>
-      </c>
-      <c r="J7" s="1">
-        <v>1.3946280165394675E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="4">
-        <v>0</v>
-      </c>
-      <c r="C8" s="1">
-        <v>9.2451191221041729E-2</v>
-      </c>
-      <c r="D8" s="1">
-        <v>9.2451191221041729E-2</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1">
-        <v>9.2451191221041729E-2</v>
-      </c>
-      <c r="G8" s="4">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1">
-        <v>9.2451191221041729E-2</v>
-      </c>
-      <c r="I8" s="1">
-        <v>0</v>
-      </c>
-      <c r="J8" s="1">
-        <v>9.2451191221041729E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="4">
-        <v>0</v>
-      </c>
-      <c r="C9" s="1">
-        <v>0.16338007724980988</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0.16338007724980988</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0.16338007724980988</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1">
-        <v>0.16338007724980988</v>
-      </c>
-      <c r="I9" s="1">
-        <v>0</v>
-      </c>
-      <c r="J9" s="1">
-        <v>0.16338007724980988</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="4">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1">
-        <v>4.9993544865259128E-4</v>
-      </c>
-      <c r="D10" s="1">
-        <v>4.9993544865259128E-4</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1">
-        <v>4.9993544865259128E-4</v>
-      </c>
-      <c r="G10" s="4">
-        <v>0.02</v>
-      </c>
-      <c r="H10" s="1">
-        <v>4.9993544865259128E-4</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="J10" s="1">
-        <v>4.9993544865259128E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="4">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1">
-        <v>3.4525200454723193E-6</v>
-      </c>
-      <c r="D11" s="1">
-        <v>3.4525200454723193E-6</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0</v>
-      </c>
-      <c r="F11" s="1">
-        <v>3.4525200454723193E-6</v>
-      </c>
-      <c r="G11" s="4">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1">
-        <v>3.4525200454723193E-6</v>
-      </c>
-      <c r="I11" s="1">
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <v>3.4525200454723193E-6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="4">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1">
-        <v>3.4682851125860878E-3</v>
-      </c>
-      <c r="D12" s="1">
-        <v>3.4682851125860878E-3</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1">
-        <v>3.4682851125860878E-3</v>
-      </c>
-      <c r="G12" s="4">
-        <v>0</v>
-      </c>
-      <c r="H12" s="1">
-        <v>3.4682851125860878E-3</v>
-      </c>
-      <c r="I12" s="1">
-        <v>0</v>
-      </c>
-      <c r="J12" s="1">
-        <v>3.4682851125860878E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="4">
-        <v>0.21</v>
-      </c>
-      <c r="C13" s="1">
-        <v>1.6017893086866013E-2</v>
-      </c>
-      <c r="D13" s="1">
-        <v>1.6017893086866013E-2</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="F13" s="1">
-        <v>1.6017893086866013E-2</v>
-      </c>
-      <c r="G13" s="4">
-        <v>0</v>
-      </c>
-      <c r="H13" s="1">
-        <v>1.6017893086866013E-2</v>
-      </c>
-      <c r="I13" s="1">
-        <v>0</v>
-      </c>
-      <c r="J13" s="1">
-        <v>1.6017893086866013E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="4">
-        <v>0.79</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0.7227845373444588</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0.72278453734445869</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0.79</v>
-      </c>
-      <c r="F14" s="1">
-        <v>0.7227845373444588</v>
-      </c>
-      <c r="G14" s="4">
-        <v>0</v>
-      </c>
-      <c r="H14" s="1">
-        <v>0.7227845373444588</v>
-      </c>
-      <c r="I14" s="1">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1">
-        <v>0.72278453734445869</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1527,10 +1020,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
@@ -1562,10 +1055,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C3" s="4">
         <v>40</v>
@@ -1597,10 +1090,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C4" s="4">
         <v>1000</v>
@@ -1632,10 +1125,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C5" s="1">
         <v>2748.0386022014691</v>
@@ -1667,10 +1160,10 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1">
         <v>79281.656703969405</v>
@@ -1702,10 +1195,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1">
         <v>91.649651416964176</v>

</xml_diff>